<commit_message>
Cleanup and improve AGENTS.md
</commit_message>
<xml_diff>
--- a/outputs/samc21-pin-allocation/samc21_pin_allocation.xlsx
+++ b/outputs/samc21-pin-allocation/samc21_pin_allocation.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2ccacb07d0b34804"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM0" sheetId="2" r:id="R5966797324fb4981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM1" sheetId="3" r:id="R7a3e89122b3c4995"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM2" sheetId="4" r:id="R2346af05269043c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STM32" sheetId="5" r:id="Reddc905ecbe44354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FTDI" sheetId="6" r:id="R4504b132092c4a49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7203cc0b85584988"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM0" sheetId="2" r:id="R6f9f200a0a5a4d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM1" sheetId="3" r:id="R2efb696a4a57481a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM2" sheetId="4" r:id="R6c8137ec712c4a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STM32" sheetId="5" r:id="R037ca390c10d46fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FTDI" sheetId="6" r:id="R11c7b9a793ea4e7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -477,14 +477,14 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>SAMC21 draft pin allocation</x:v>
+        <x:v>Board 1 draft pin allocation</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str"/>
       <x:c r="C1" s="6" t="str"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Board 1 · ATSAMC21G17A-AUT ×3 · 2026-09-06</x:v>
+        <x:v>Board 1 · gateway, three leaves, FTDI and EEPROM · notes reconciled 2026-09-07</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str"/>
       <x:c r="C2" s="6" t="str"/>
@@ -505,10 +505,10 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>48 physical pads for each leaf. All assignments proposed and evidence unverified. No CAD or hardware validation.</x:v>
+        <x:v>264 pad rows: SAMs 3 × 48, STM32 64, FTDI 48 and EEPROM 8. All allocations remain unverified; no Board 1 CAD exists.</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
-        <x:v>B1-R001; B1-Q005; USR-19</x:v>
+        <x:v>B1-R001/005; B1-Q002/005/012; ADR-004/018</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
@@ -549,10 +549,10 @@
         <x:v>Multidrop circuit</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>TX and RX are separate logical reservations. External open-drain drive/sense circuitry, idle polarity and reset behavior must be designed before connection.</x:v>
+        <x:v>ADR-033/039 select the second LV125 and pulls: TX to /OE, A to GND, Y to UART_MD; RX senses the bus. Reset/ramp behavior and rate remain unqualified.</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
-        <x:v>B1-Q003</x:v>
+        <x:v>ADR-033/039; B1-Q003/005</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -560,10 +560,10 @@
         <x:v>Clock</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>PA14/PA15 pads23/24 are XIN/XOUT. Selected MCU crystal: ECS-120-20-3X-EN-TR. CL 20 pF is crystal load, not the individual capacitor value.</x:v>
+        <x:v>PA14/PA15 pads23/24 are XIN/XOUT. Leaf crystal and initial load capacitors are accepted; see B1-B020/043. Startup/drive/loading remain B1-Q008.</x:v>
       </x:c>
       <x:c r="C9" s="3" t="str">
-        <x:v>ADR-014; B1-Q008</x:v>
+        <x:v>ADR-014/030/031; B1-Q008</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -571,10 +571,10 @@
         <x:v>Debug</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>PA30 pad45 SWCLK; PA31 pad46 SWDIO; pad40 RESET. Individual 10-pin Cortex SWD header per leaf; exact header and adapter wiring TBD.</x:v>
+        <x:v>PA30/pad45 SWCLK; PA31/pad46 SWDIO; pad40 RESET. SWD header MPN B1-B009 is accepted; numbering, footprint and probe/cable compatibility remain open.</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
-        <x:v>ADR-011; B1-Q004/005</x:v>
+        <x:v>ADR-011; ADR-026 (026-reva-connectors.md); B1-Q004/005</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -582,10 +582,10 @@
         <x:v>GPIO / LED</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
-        <x:v>Four proposed breakouts: PA02, PA03, PB08, PB09. LED PA27. Exact LED current and breakout load/protection remain TBD.</x:v>
+        <x:v>Four GPIOs per MCU and LED/resistor parts are accepted. Leaf pad choices PA02/PA03/PB08/PB09 and LED PA27 remain draft; load/protection and LED drive need review.</x:v>
       </x:c>
       <x:c r="C11" s="3" t="str">
-        <x:v>B1-R019/020; B1-Q010</x:v>
+        <x:v>ADR-029/039; B1-R019/020; B1-Q005/010</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -593,10 +593,10 @@
         <x:v>Power</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
-        <x:v>3.3 V system intended for VDDIN, VDDIO and VDDANA. VDDCORE is regulator output for its local capacitor only, never tied to 3V3_SYS.</x:v>
+        <x:v>VDDIN/VDDIO/VDDANA use 3V3_SYS. Each VDDCORE has its own accepted ceramic capacitor pair B1-B040/041; never join core outputs or tie them to 3V3_SYS.</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
-        <x:v>DS60001479J, §7; ADR-010; B1-Q002/005</x:v>
+        <x:v>ADR-010; ADR-026 (026-sam-core-ceramic.md); ADR-027; B1-Q002/005/011</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
@@ -659,10 +659,10 @@
         <x:v>Crystal source</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
-        <x:v>ECS CSM-3X Rev.2017. Smaller crystal remains unverified for MCU startup/drive. Separate accurate FT232HL crystal candidate recorded in project notes.</x:v>
+        <x:v>MCU and separate FTDI crystals are finalized; initial load capacitors are accepted. B1-B014/019/020/042/043/058 own the parts; oscillator qualification remains open.</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
-        <x:v>https://ecsxtal.com/store/pdf/CSM-3X.pdf</x:v>
+        <x:v>ADR-014/017/030/031; B1-Q008; https://ecsxtal.com/store/pdf/CSM-3X.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
@@ -670,10 +670,10 @@
         <x:v>Stable IDs</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
-        <x:v>SAM0 B1-P025–072; SAM1 B1-P073–120; SAM2 B1-P121–168. Parent resource rows retained. Blank parent is represented by NA.</x:v>
+        <x:v>SAM0 B1-P025–072; SAM1 B1-P073–120; SAM2 B1-P121–168; STM32 B1-P169–232; FTDI/EEPROM B1-P233–288. Parent groups B1-P001–024 retained.</x:v>
       </x:c>
       <x:c r="C19" s="3" t="str">
-        <x:v>Board 1 pinmap; next unused ID B1-P169</x:v>
+        <x:v>Board 1 pinmap; next unused ID B1-P289</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -681,10 +681,10 @@
         <x:v>Editing</x:v>
       </x:c>
       <x:c r="B20" s="3" t="str">
-        <x:v>Signal/peripheral/mux entries are draft choices. Changing them requires a fresh mux and physical connectivity review. Source references do not mean verified.</x:v>
+        <x:v>Notes reflect ADR-039 baseline. Signal/peripheral/mux choices remain draft. Source citations and accepted MPNs do not establish electrical verification.</x:v>
       </x:c>
       <x:c r="C20" s="3" t="str">
-        <x:v>B1-Q005</x:v>
+        <x:v>B1-Q005; Board 1 unfinished implementation decisions</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1322,7 +1322,7 @@
         <x:v>B1-R003</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
-        <x:v>To external open-drain interface TBD. Do not connect push-pull TX directly to shared bus. TXPO=0.</x:v>
+        <x:v>To B1-B066 LV125 /OE; A=GND, Y=UART_MD (ADR-033). /OE pull-up B1-B008 accepted ADR-039. TXPO=0; reset/ramp/timing unverified.</x:v>
       </x:c>
       <x:c r="K17" s="3" t="str">
         <x:v>DS60001479J p.22; 30; 505</x:v>
@@ -1363,7 +1363,7 @@
         <x:v>B1-R003</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>Sense UART_MD through interface TBD. RXPO=1. Rate/pull-up pending B1-Q003.</x:v>
+        <x:v>Sense shared UART_MD; RXPO=1. Bus pull-up B1-B074 accepted ADR-039. Rate, thresholds and rise time remain B1-Q003/005.</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
         <x:v>DS60001479J p.22; 30; 505</x:v>
@@ -1732,7 +1732,7 @@
         <x:v>B1-R015</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
-        <x:v>ECS-120-20-3X-EN-TR, 12 MHz. CL=20 pF. Load network/startup/drive TBD.</x:v>
+        <x:v>Selected 12 MHz MCU crystal B1-B020; initial load caps B1-B043 accepted ADR-031. Startup, drive and loading remain B1-Q008.</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str">
         <x:v>DS60001479J p.22; 34; 191–192</x:v>
@@ -2388,7 +2388,7 @@
         <x:v>B1-R019</x:v>
       </x:c>
       <x:c r="J43" s="3" t="str">
-        <x:v>Proposed active-high LED. Resistor/current TBD; not counted as spare GPIO.</x:v>
+        <x:v>PA27 LED drive remains proposed. LED and resistor B1-B024/026 accepted ADR-029/039; current/visibility remain B1-Q010.</x:v>
       </x:c>
       <x:c r="K43" s="3" t="str">
         <x:v>DS60001479J p.22; 30</x:v>
@@ -2552,7 +2552,7 @@
         <x:v>B1-R001</x:v>
       </x:c>
       <x:c r="J47" s="3" t="str">
-        <x:v>Regulator output. Local core capacitor only; value per decoupling review. Do not tie to 3.3 V.</x:v>
+        <x:v>Separate regulator output; accepted ceramic pair B1-B040/041, ADR-026 (026-sam-core-ceramic.md)/027. Never join core rails or 3V3_SYS; qualify stability.</x:v>
       </x:c>
       <x:c r="K47" s="3" t="str">
         <x:v>DS60001479J p.22; §7</x:v>
@@ -2776,7 +2776,7 @@
       <x:c r="B55" s="1"/>
       <x:c r="C55" s="1"/>
       <x:c r="D55" s="1" t="str">
-        <x:v>B1-R025 / ADR-032: dedicated 115200 baud; 8N1, no flow control proposed. 1x3 2.54 mm header: 1=MCU TX, 2=MCU RX, 3=GND. No VCC pin. B1-B059/060; B1-Q014.</x:v>
+        <x:v>ADR-032/039: dedicated 115200-baud debug; 1x3 cut header B1-B059 from strip B1-B027. Proposed order 1=MCU TX, 2=MCU RX, 3=GND; 8N1/no flow control. Off-state support B1-B060 remains TBD.</x:v>
       </x:c>
       <x:c r="E55" s="1"/>
       <x:c r="F55" s="1"/>
@@ -2799,7 +2799,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf562bce6464b42ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4be5644386b6422b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3434,7 +3434,7 @@
         <x:v>B1-R003</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
-        <x:v>To external open-drain interface TBD. Do not connect push-pull TX directly to shared bus. TXPO=0.</x:v>
+        <x:v>To B1-B066 LV125 /OE; A=GND, Y=UART_MD (ADR-033). /OE pull-up B1-B008 accepted ADR-039. TXPO=0; reset/ramp/timing unverified.</x:v>
       </x:c>
       <x:c r="K17" s="3" t="str">
         <x:v>DS60001479J p.22; 30; 505</x:v>
@@ -3475,7 +3475,7 @@
         <x:v>B1-R003</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>Sense UART_MD through interface TBD. RXPO=1. Rate/pull-up pending B1-Q003.</x:v>
+        <x:v>Sense shared UART_MD; RXPO=1. Bus pull-up B1-B074 accepted ADR-039. Rate, thresholds and rise time remain B1-Q003/005.</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
         <x:v>DS60001479J p.22; 30; 505</x:v>
@@ -3844,7 +3844,7 @@
         <x:v>B1-R015</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
-        <x:v>ECS-120-20-3X-EN-TR, 12 MHz. CL=20 pF. Load network/startup/drive TBD.</x:v>
+        <x:v>Selected 12 MHz MCU crystal B1-B020; initial load caps B1-B043 accepted ADR-031. Startup, drive and loading remain B1-Q008.</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str">
         <x:v>DS60001479J p.22; 34; 191–192</x:v>
@@ -4500,7 +4500,7 @@
         <x:v>B1-R019</x:v>
       </x:c>
       <x:c r="J43" s="3" t="str">
-        <x:v>Proposed active-high LED. Resistor/current TBD; not counted as spare GPIO.</x:v>
+        <x:v>PA27 LED drive remains proposed. LED and resistor B1-B024/026 accepted ADR-029/039; current/visibility remain B1-Q010.</x:v>
       </x:c>
       <x:c r="K43" s="3" t="str">
         <x:v>DS60001479J p.22; 30</x:v>
@@ -4664,7 +4664,7 @@
         <x:v>B1-R001</x:v>
       </x:c>
       <x:c r="J47" s="3" t="str">
-        <x:v>Regulator output. Local core capacitor only; value per decoupling review. Do not tie to 3.3 V.</x:v>
+        <x:v>Separate regulator output; accepted ceramic pair B1-B040/041, ADR-026 (026-sam-core-ceramic.md)/027. Never join core rails or 3V3_SYS; qualify stability.</x:v>
       </x:c>
       <x:c r="K47" s="3" t="str">
         <x:v>DS60001479J p.22; §7</x:v>
@@ -4888,7 +4888,7 @@
       <x:c r="B55" s="1"/>
       <x:c r="C55" s="1"/>
       <x:c r="D55" s="1" t="str">
-        <x:v>B1-R025 / ADR-032: dedicated 115200 baud; 8N1, no flow control proposed. 1x3 2.54 mm header: 1=MCU TX, 2=MCU RX, 3=GND. No VCC pin. B1-B059/060; B1-Q014.</x:v>
+        <x:v>ADR-032/039: dedicated 115200-baud debug; 1x3 cut header B1-B059 from strip B1-B027. Proposed order 1=MCU TX, 2=MCU RX, 3=GND; 8N1/no flow control. Off-state support B1-B060 remains TBD.</x:v>
       </x:c>
       <x:c r="E55" s="1"/>
       <x:c r="F55" s="1"/>
@@ -4911,7 +4911,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R375edd2720584c9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55fd92f26cef41fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5546,7 +5546,7 @@
         <x:v>B1-R003</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
-        <x:v>To external open-drain interface TBD. Do not connect push-pull TX directly to shared bus. TXPO=0.</x:v>
+        <x:v>To B1-B066 LV125 /OE; A=GND, Y=UART_MD (ADR-033). /OE pull-up B1-B008 accepted ADR-039. TXPO=0; reset/ramp/timing unverified.</x:v>
       </x:c>
       <x:c r="K17" s="3" t="str">
         <x:v>DS60001479J p.22; 30; 505</x:v>
@@ -5587,7 +5587,7 @@
         <x:v>B1-R003</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>Sense UART_MD through interface TBD. RXPO=1. Rate/pull-up pending B1-Q003.</x:v>
+        <x:v>Sense shared UART_MD; RXPO=1. Bus pull-up B1-B074 accepted ADR-039. Rate, thresholds and rise time remain B1-Q003/005.</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
         <x:v>DS60001479J p.22; 30; 505</x:v>
@@ -5956,7 +5956,7 @@
         <x:v>B1-R015</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
-        <x:v>ECS-120-20-3X-EN-TR, 12 MHz. CL=20 pF. Load network/startup/drive TBD.</x:v>
+        <x:v>Selected 12 MHz MCU crystal B1-B020; initial load caps B1-B043 accepted ADR-031. Startup, drive and loading remain B1-Q008.</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str">
         <x:v>DS60001479J p.22; 34; 191–192</x:v>
@@ -6612,7 +6612,7 @@
         <x:v>B1-R019</x:v>
       </x:c>
       <x:c r="J43" s="3" t="str">
-        <x:v>Proposed active-high LED. Resistor/current TBD; not counted as spare GPIO.</x:v>
+        <x:v>PA27 LED drive remains proposed. LED and resistor B1-B024/026 accepted ADR-029/039; current/visibility remain B1-Q010.</x:v>
       </x:c>
       <x:c r="K43" s="3" t="str">
         <x:v>DS60001479J p.22; 30</x:v>
@@ -6776,7 +6776,7 @@
         <x:v>B1-R001</x:v>
       </x:c>
       <x:c r="J47" s="3" t="str">
-        <x:v>Regulator output. Local core capacitor only; value per decoupling review. Do not tie to 3.3 V.</x:v>
+        <x:v>Separate regulator output; accepted ceramic pair B1-B040/041, ADR-026 (026-sam-core-ceramic.md)/027. Never join core rails or 3V3_SYS; qualify stability.</x:v>
       </x:c>
       <x:c r="K47" s="3" t="str">
         <x:v>DS60001479J p.22; §7</x:v>
@@ -7000,7 +7000,7 @@
       <x:c r="B55" s="1"/>
       <x:c r="C55" s="1"/>
       <x:c r="D55" s="1" t="str">
-        <x:v>B1-R025 / ADR-032: dedicated 115200 baud; 8N1, no flow control proposed. 1x3 2.54 mm header: 1=MCU TX, 2=MCU RX, 3=GND. No VCC pin. B1-B059/060; B1-Q014.</x:v>
+        <x:v>ADR-032/039: dedicated 115200-baud debug; 1x3 cut header B1-B059 from strip B1-B027. Proposed order 1=MCU TX, 2=MCU RX, 3=GND; 8N1/no flow control. Off-state support B1-B060 remains TBD.</x:v>
       </x:c>
       <x:c r="E55" s="1"/>
       <x:c r="F55" s="1"/>
@@ -7023,7 +7023,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78cea3c1951d45d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf988dcbbc324ad8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7330,7 +7330,7 @@
         <x:v>B1-R015</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>12 MHz ECS-120-20-3X-EN-TR. CL=20 pF; individual capacitors TBD.</x:v>
+        <x:v>Selected 12 MHz MCU crystal B1-B019; initial load caps B1-B042 accepted ADR-031. Startup, drive and loading remain B1-Q008.</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
         <x:v>DS12288 Rev.6 p.50; 58</x:v>
@@ -8027,7 +8027,7 @@
         <x:v>B1-R019</x:v>
       </x:c>
       <x:c r="J26" s="3" t="str">
-        <x:v>Proposed active-high LED; resistor/current TBD. Not counted as spare GPIO.</x:v>
+        <x:v>PA5 LED drive remains proposed. LED and resistor B1-B024/026 accepted ADR-029/039; current/visibility remain B1-Q010.</x:v>
       </x:c>
       <x:c r="K26" s="3" t="str">
         <x:v>DS12288 Rev.6 p.50; 60</x:v>
@@ -8888,7 +8888,7 @@
         <x:v>B1-R003</x:v>
       </x:c>
       <x:c r="J47" s="3" t="str">
-        <x:v>To open-drain interface TBD. Do not connect push-pull TX directly to shared UART_MD.</x:v>
+        <x:v>To B1-B066 LV125 /OE; A=GND, Y=UART_MD (ADR-033). /OE pull-up B1-B008 accepted ADR-039. Reset/ramp/timing remain unverified.</x:v>
       </x:c>
       <x:c r="K47" s="3" t="str">
         <x:v>DS12288 Rev.6 p.50; 65–66; 73</x:v>
@@ -8929,7 +8929,7 @@
         <x:v>B1-R003</x:v>
       </x:c>
       <x:c r="J48" s="3" t="str">
-        <x:v>Sense shared UART_MD through circuit TBD. Exact rate and idle/reset behavior pending.</x:v>
+        <x:v>Sense shared UART_MD with accepted B1-B074 bus pull-up (ADR-039). Rate, thresholds and idle/reset behavior remain B1-Q003/005.</x:v>
       </x:c>
       <x:c r="K48" s="3" t="str">
         <x:v>DS12288 Rev.6 p.50; 66; 73</x:v>
@@ -9257,7 +9257,7 @@
         <x:v>B1-R016; B1-R021</x:v>
       </x:c>
       <x:c r="J56" s="3" t="str">
-        <x:v>To RS-485 PHY driver input. 12 Mbps ceiling; exact PHY/timing pending B1-Q009.</x:v>
+        <x:v>To selected ST3485EBDR DI. 12 Mbps ceiling retained; actual rate, control timing and remote kit compatibility remain B1-Q009.</x:v>
       </x:c>
       <x:c r="K56" s="3" t="str">
         <x:v>DS12288 Rev.6 p.50; 67; 75</x:v>
@@ -9806,7 +9806,7 @@
       <x:c r="B73" s="1"/>
       <x:c r="C73" s="1"/>
       <x:c r="D73" s="1" t="str">
-        <x:v>Keep PG10 as NRST and PA13/PA14 as SWD. PB8 reserved for BOOT0. Option bytes, probe header/adapter and reset pulls remain B1-Q004/005. SWO is not allocated.</x:v>
+        <x:v>Keep NRST and SWD. ADR-023 allocates CBUS5 to NRST and CBUS6 to BOOT0 through B1-B053 interfaces TBD. Defaults: reset released, BOOT0 low. Option bytes, pulls and probe compatibility remain B1-Q004/005/013.</x:v>
       </x:c>
       <x:c r="E73" s="1"/>
       <x:c r="F73" s="1"/>
@@ -9939,7 +9939,7 @@
       <x:c r="B80" s="1"/>
       <x:c r="C80" s="1"/>
       <x:c r="D80" s="1" t="str">
-        <x:v>B1-P169–B1-P232. B1-P001–006 remain parent groups. RS-485, LED and GPIO rows use requirement references directly. Next pin ID B1-P233.</x:v>
+        <x:v>STM32 B1-P169–232; B1-P001–006 remain parent groups. FTDI/EEPROM use B1-P233–288. Next unused pin ID B1-P289.</x:v>
       </x:c>
       <x:c r="E80" s="1"/>
       <x:c r="F80" s="1"/>
@@ -9958,7 +9958,7 @@
       <x:c r="B83" s="1"/>
       <x:c r="C83" s="1"/>
       <x:c r="D83" s="1" t="str">
-        <x:v>B1-R025 / ADR-032: dedicated 115200 baud; 8N1, no flow control proposed. 1x3 2.54 mm header: 1=MCU TX, 2=MCU RX, 3=GND. No VCC pin. B1-B059/060; B1-Q014.</x:v>
+        <x:v>ADR-032/039: dedicated 115200-baud debug; 1x3 cut header B1-B059 from strip B1-B027. Proposed order 1=MCU TX, 2=MCU RX, 3=GND; 8N1/no flow control. Off-state support B1-B060 remains TBD.</x:v>
       </x:c>
       <x:c r="E83" s="1"/>
       <x:c r="F83" s="1"/>
@@ -9973,7 +9973,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31280dbb229e4ac8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fbca177992f4d36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10116,7 +10116,7 @@
         <x:v>B1-R005</x:v>
       </x:c>
       <x:c r="J5" s="3" t="str">
-        <x:v>12 MHz B1-B014 candidate per ADR-017. Load capacitors TBD; total accuracy within 30 ppm.</x:v>
+        <x:v>FTDI crystal B1-B014 finalized ADR-030; initial load caps B1-B058 accepted ADR-031. Loading, startup, drive and frequency remain B1-Q008.</x:v>
       </x:c>
       <x:c r="K5" s="3" t="str">
         <x:v>FT_000288 v2.2 p.11; 48</x:v>
@@ -10280,7 +10280,7 @@
         <x:v>B1-R005</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>12 kohm 1% resistor to GND. 0805 proposed; exact resistor in B1-B017 TBD.</x:v>
+        <x:v>Accepted REF resistor B1-B057: 12 kohm 1% to GND (ADR-031). Footprint and circuit qualification remain B1-Q002.</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
         <x:v>FT_000288 v2.2 p.11</x:v>
@@ -10567,7 +10567,7 @@
         <x:v>B1-R012</x:v>
       </x:c>
       <x:c r="J16" s="3" t="str">
-        <x:v>Connect to independent VCCD 3.3 V output. All three VCCIO pins required; local bypass B1-B017.</x:v>
+        <x:v>Independent VCCD supply; all three VCCIO pins required. Accepted bypass MPNs B1-B061–063; counts/rail allocation remain B1-Q002.</x:v>
       </x:c>
       <x:c r="K16" s="3" t="str">
         <x:v>FT_000288 v2.2 p.11; 45</x:v>
@@ -10936,7 +10936,7 @@
         <x:v>B1-R012</x:v>
       </x:c>
       <x:c r="J25" s="3" t="str">
-        <x:v>ACBUS0 proposed. To always-powered default-off polarity interface for SC189 EN, per ADR-013.</x:v>
+        <x:v>PWREN# to MC74HC1G14DBVT1G, then TPS560430 EN (ADR-021/024). Pulls B1-B054/055 accepted; startup/default-off qualification remains B1-Q002.</x:v>
       </x:c>
       <x:c r="K25" s="3" t="str">
         <x:v>FT_000288 v2.2 p.12–13</x:v>
@@ -11059,7 +11059,7 @@
         <x:v>B1-R012</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
-        <x:v>Connect to independent VCCD 3.3 V output. All three VCCIO pins required; local bypass B1-B017.</x:v>
+        <x:v>Independent VCCD supply; all three VCCIO pins required. Accepted bypass MPNs B1-B061–063; counts/rail allocation remain B1-Q002.</x:v>
       </x:c>
       <x:c r="K28" s="3" t="str">
         <x:v>FT_000288 v2.2 p.11; 45</x:v>
@@ -11469,7 +11469,7 @@
         <x:v>B1-R005; B1-R012</x:v>
       </x:c>
       <x:c r="J38" s="3" t="str">
-        <x:v>Independent bridge reset. Pull-up/RC or supervisor TBD under B1-Q002; allow EEPROM startup before read.</x:v>
+        <x:v>RESET# uses accepted pull-up B1-B051 and capacitor B1-B064 (ADR-022/027/028). No external supervisor. EEPROM startup/ramp checks B1-Q002/012.</x:v>
       </x:c>
       <x:c r="K38" s="3" t="str">
         <x:v>FT_000288 v2.2 p.11; §4.11</x:v>
@@ -11715,7 +11715,7 @@
         <x:v>B1-R012</x:v>
       </x:c>
       <x:c r="J44" s="3" t="str">
-        <x:v>From USB-B protected supply before SC189. Local bypass/inrush budget B1-B017/B1-Q002.</x:v>
+        <x:v>From ramped USB_5V after TPS22810, shared with buck VIN (ADR-021/022). USB_5V_PROTECTED is this workbook alias. Bypass counts B1-B061–063 TBD.</x:v>
       </x:c>
       <x:c r="K44" s="3" t="str">
         <x:v>FT_000288 v2.2 p.11; 45</x:v>
@@ -11838,7 +11838,7 @@
         <x:v>B1-R005; B1-R012</x:v>
       </x:c>
       <x:c r="J47" s="3" t="str">
-        <x:v>Direct to EEPROM DI/pad 3; DO/pad 4 through 2.2 kohm. DO side has 10 kohm pull-up to 3V3_FTDI.</x:v>
+        <x:v>EEDATA to EEPROM DI directly; DO via accepted B1-B056; DO-side pull-up B1-B065 to 3V3_FTDI. ADR-028/030; timing/startup remain B1-Q012.</x:v>
       </x:c>
       <x:c r="K47" s="3" t="str">
         <x:v>FT_000288 v2.2 p.12; 49 Fig.7.1</x:v>
@@ -11961,7 +11961,7 @@
         <x:v>B1-R012</x:v>
       </x:c>
       <x:c r="J50" s="3" t="str">
-        <x:v>Connect to independent VCCD 3.3 V output. All three VCCIO pins required; local bypass B1-B017.</x:v>
+        <x:v>Independent VCCD supply; all three VCCIO pins required. Accepted bypass MPNs B1-B061–063; counts/rail allocation remain B1-Q002.</x:v>
       </x:c>
       <x:c r="K50" s="3" t="str">
         <x:v>FT_000288 v2.2 p.11; 45</x:v>
@@ -12310,7 +12310,7 @@
         <x:v>B1-R005; B1-R012</x:v>
       </x:c>
       <x:c r="J61" s="3" t="str">
-        <x:v>To EEDATA through 2.2 kohm; 10 kohm pull-up on DO side to 3V3_FTDI.</x:v>
+        <x:v>DO to EEDATA via accepted B1-B056; DO-side pull-up B1-B065 to 3V3_FTDI. ADR-028/030; timing remains B1-Q012.</x:v>
       </x:c>
       <x:c r="K61" s="3" t="str">
         <x:v>DS20006260B p.3–9; 31</x:v>
@@ -12474,7 +12474,7 @@
         <x:v>B1-R005; B1-R012</x:v>
       </x:c>
       <x:c r="J65" s="3" t="str">
-        <x:v>From FT232HL VCCD/pad 39. Propose 100 nF local 0805 bypass in B1-B017. Startup constraints B1-Q012.</x:v>
+        <x:v>From FT232HL VCCD. Local bypass belongs to accepted B1-B061 allocation; final count and startup constraints remain B1-Q002/012.</x:v>
       </x:c>
       <x:c r="K65" s="3" t="str">
         <x:v>DS20006260B p.3–9; 31</x:v>
@@ -12531,7 +12531,7 @@
       <x:c r="B70" s="1"/>
       <x:c r="C70" s="1"/>
       <x:c r="D70" s="1" t="str">
-        <x:v>Program/read back EEPROM, then re-enumerate. Blank or corrupt EEPROM must leave SC189 EN off. Pull-down-in-suspend policy and receiver pulls require review.</x:v>
+        <x:v>Program/read back and re-enumerate. Blank/corrupt EEPROM must keep TPS560430 EN off through the accepted inverter/pulls. Suspend defaults and receiver pulls remain B1-Q002.</x:v>
       </x:c>
       <x:c r="E70" s="1"/>
       <x:c r="F70" s="1"/>
@@ -12588,7 +12588,7 @@
       <x:c r="B73" s="1"/>
       <x:c r="C73" s="1"/>
       <x:c r="D73" s="1" t="str">
-        <x:v>EEPROM and FTDI bypass/filter parts belong to B1-B017, separate from main-rail capacitance. VCCA and VCORE each have their own 100 nF only.</x:v>
+        <x:v>Bridge caps B1-B061–063 have accepted MPNs but TBD counts; split support B1-B051/054–058/064/065 is excluded from residual B1-B017. 3V3_FTDI aliases FTDI_3V3; VCCA/VCORE stay separate.</x:v>
       </x:c>
       <x:c r="E73" s="1"/>
       <x:c r="F73" s="1"/>
@@ -12626,7 +12626,7 @@
       <x:c r="B75" s="1"/>
       <x:c r="C75" s="1"/>
       <x:c r="D75" s="1" t="str">
-        <x:v>B1-Q002/008/012: power, default-off logic, SN74LV125 logic levels and 12 Mbaud timing, crystal, EEPROM startup/clock, exact support parts and footprints. No ERC/DRC or bench validation.</x:v>
+        <x:v>B1-Q002/008/012/013: rails, enables/defaults, VCP timing, oscillator/EEPROM qualification and CBUS interfaces. Selected parts remain accepted; all pad evidence stays unverified.</x:v>
       </x:c>
       <x:c r="E75" s="1"/>
       <x:c r="F75" s="1"/>
@@ -12679,8 +12679,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R721a2ff0085746ed"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R850ee3d52e964b21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7559dc01174432"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eeac784a8cc4dcd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>